<commit_message>
Laminas regeneradas (regeneracion completa del 2026-10-04), piramides 2018-2024, empates nombrados (#191) (graficos_regionales_correlaciones)
</commit_message>
<xml_diff>
--- a/output/graficos_regionales_correlaciones/plot_regional_correl_matriz_d_otrasrel_a_2020_o_higgins.xlsx
+++ b/output/graficos_regionales_correlaciones/plot_regional_correl_matriz_d_otrasrel_a_2020_o_higgins.xlsx
@@ -132,7 +132,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-10-01 23:20</t>
+    <t xml:space="preserve">2026-10-05 19:43</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>
@@ -1165,7 +1165,7 @@
         <v>16</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>-0.22</v>
+        <v>-0.21</v>
       </c>
       <c r="F28" s="2" t="n">
         <v>-0.07</v>

</xml_diff>